<commit_message>
Índices oficiais do BCB (INPC, IGP-DI, IPCA-E, SELIC) até 08/2026 e importação de CSV do SGS
INPC acumulado de 2015 a 2025 confere com os reajustes do INSS; SELIC 12/2021-04/2025
confere com o cálculo-modelo (39,21%).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZmLqeaMLjqa4f3gXsmFk8
</commit_message>
<xml_diff>
--- a/exemplos/Calculo_CNIS_ficticio.xlsx
+++ b/exemplos/Calculo_CNIS_ficticio.xlsx
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>0.4</v>
+        <v>0.19</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>1</v>
+        <v>0.83</v>
       </c>
       <c r="D4" s="18" t="n"/>
     </row>
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1</v>
+        <v>0.89</v>
       </c>
       <c r="D5" s="18" t="n"/>
     </row>
@@ -1197,10 +1197,10 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>0.4</v>
+        <v>0.46</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1</v>
+        <v>0.83</v>
       </c>
       <c r="D6" s="18" t="n"/>
     </row>
@@ -1211,10 +1211,10 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>1</v>
+        <v>0.79</v>
       </c>
       <c r="D7" s="18" t="n"/>
     </row>
@@ -1225,10 +1225,10 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>0.4</v>
+        <v>0.26</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>1</v>
+        <v>0.91</v>
       </c>
       <c r="D8" s="18" t="n"/>
     </row>
@@ -1239,10 +1239,10 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>0.4</v>
+        <v>-0.14</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>1</v>
+        <v>0.87</v>
       </c>
       <c r="D9" s="18" t="n"/>
     </row>
@@ -1253,10 +1253,10 @@
         </is>
       </c>
       <c r="B10" s="18" t="n">
-        <v>0.4</v>
+        <v>0.48</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>1</v>
+        <v>0.84</v>
       </c>
       <c r="D10" s="18" t="n"/>
     </row>
@@ -1267,10 +1267,10 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>0.4</v>
+        <v>0.61</v>
       </c>
       <c r="C11" s="18" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="D11" s="18" t="n"/>
     </row>
@@ -1281,10 +1281,10 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>1</v>
+        <v>0.79</v>
       </c>
       <c r="D12" s="18" t="n"/>
     </row>
@@ -1295,10 +1295,10 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>0.4</v>
+        <v>0.48</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
       <c r="D13" s="18" t="n"/>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B14" s="18" t="n"/>
       <c r="C14" s="18" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="D14" s="18" t="n"/>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B15" s="18" t="n"/>
       <c r="C15" s="18" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="D15" s="18" t="n"/>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B16" s="18" t="n"/>
       <c r="C16" s="18" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="D16" s="18" t="n"/>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B17" s="18" t="n"/>
       <c r="C17" s="18" t="n">
-        <v>1</v>
+        <v>1.06</v>
       </c>
       <c r="D17" s="18" t="n"/>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B18" s="18" t="n"/>
       <c r="C18" s="18" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="D18" s="18" t="n"/>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="B19" s="18" t="n"/>
       <c r="C19" s="18" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="D19" s="18" t="n"/>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="B20" s="18" t="n"/>
       <c r="C20" s="18" t="n">
-        <v>1</v>
+        <v>1.28</v>
       </c>
       <c r="D20" s="18" t="n"/>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="B21" s="18" t="n"/>
       <c r="C21" s="18" t="n">
-        <v>1</v>
+        <v>1.16</v>
       </c>
       <c r="D21" s="18" t="n"/>
     </row>
@@ -1405,13 +1405,13 @@
         </is>
       </c>
       <c r="B22" s="18" t="n">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>1</v>
+        <v>1.22</v>
       </c>
       <c r="D22" s="18" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="23">
@@ -1421,13 +1421,13 @@
         </is>
       </c>
       <c r="B23" s="18" t="n">
-        <v>0.4</v>
+        <v>0.03</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>1</v>
+        <v>1.28</v>
       </c>
       <c r="D23" s="18" t="n">
-        <v>0.6</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="24">
@@ -1437,13 +1437,13 @@
         </is>
       </c>
       <c r="B24" s="18" t="n">
-        <v>0.4</v>
+        <v>0.03</v>
       </c>
       <c r="C24" s="18" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="D24" s="18" t="n">
-        <v>0.6</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="25">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="B25" s="18" t="n">
-        <v>0.4</v>
+        <v>0.21</v>
       </c>
       <c r="C25" s="18" t="n">
-        <v>1</v>
+        <v>1.22</v>
       </c>
       <c r="D25" s="18" t="n">
-        <v>0.6</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="26">
@@ -1469,13 +1469,13 @@
         </is>
       </c>
       <c r="B26" s="18" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="C26" s="18" t="n">
-        <v>1</v>
+        <v>1.16</v>
       </c>
       <c r="D26" s="18" t="n">
-        <v>0.6</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="27">
@@ -1485,13 +1485,13 @@
         </is>
       </c>
       <c r="B27" s="18" t="n">
-        <v>0.4</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C27" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="18" t="n">
-        <v>0.6</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="28">
@@ -1501,13 +1501,13 @@
         </is>
       </c>
       <c r="B28" s="18" t="n">
-        <v>0.4</v>
+        <v>0.91</v>
       </c>
       <c r="C28" s="18" t="n">
-        <v>1</v>
+        <v>1.21</v>
       </c>
       <c r="D28" s="18" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="29">
@@ -1517,13 +1517,13 @@
         </is>
       </c>
       <c r="B29" s="18" t="n">
-        <v>0.4</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C29" s="18" t="n">
-        <v>1</v>
+        <v>1.09</v>
       </c>
       <c r="D29" s="18" t="n">
-        <v>0.6</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="30">
@@ -1533,13 +1533,13 @@
         </is>
       </c>
       <c r="B30" s="18" t="n">
-        <v>0.4</v>
+        <v>0.65</v>
       </c>
       <c r="C30" s="18" t="n">
-        <v>1</v>
+        <v>1.07</v>
       </c>
       <c r="D30" s="18" t="n">
-        <v>0.6</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="31">
@@ -1549,13 +1549,13 @@
         </is>
       </c>
       <c r="B31" s="18" t="n">
-        <v>0.4</v>
+        <v>0.14</v>
       </c>
       <c r="C31" s="18" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="D31" s="18" t="n">
-        <v>0.6</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="32">
@@ -1565,13 +1565,13 @@
         </is>
       </c>
       <c r="B32" s="18" t="n">
-        <v>0.4</v>
+        <v>-0.01</v>
       </c>
       <c r="C32" s="18" t="n">
-        <v>1</v>
+        <v>1.22</v>
       </c>
       <c r="D32" s="18" t="n">
-        <v>0.6</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="33">
@@ -1581,13 +1581,13 @@
         </is>
       </c>
       <c r="B33" s="18" t="n">
-        <v>0.4</v>
+        <v>-0.32</v>
       </c>
       <c r="C33" s="18" t="n">
-        <v>1</v>
+        <v>1.09</v>
       </c>
       <c r="D33" s="18" t="n">
-        <v>0.6</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="35">
@@ -1608,7 +1608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -1631,19 +1631,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>• reajuste de 2026 (3.9%) não foi conferido na fonte oficial</t>
+          <t>• salario_minimo de 2026-01 (1621.0) não foi conferido na fonte oficial</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
-        <is>
-          <t>• salario_minimo de 2026-01 (1621.0) não foi conferido na fonte oficial</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
         <is>
           <t>• teto de 2026-01 (8475.55) não foi conferido na fonte oficial</t>
         </is>
@@ -12069,7 +12062,7 @@
         <v/>
       </c>
       <c r="C20" s="17" t="n">
-        <v>4.07</v>
+        <v>3.34</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>8157.41</v>
@@ -13040,7 +13033,7 @@
         <v/>
       </c>
       <c r="J16" s="10" t="n">
-        <v>18</v>
+        <v>17.31</v>
       </c>
       <c r="K16" s="4">
         <f>ROUND(I16*J16/100,2)</f>
@@ -13051,14 +13044,14 @@
         <v/>
       </c>
       <c r="M16" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N16" s="4">
         <f>ROUND(L16*M16,2)</f>
         <v/>
       </c>
       <c r="O16" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P16" s="4">
         <f>ROUND(N16*O16/100,2)</f>
@@ -13121,7 +13114,7 @@
         <v/>
       </c>
       <c r="J17" s="10" t="n">
-        <v>17</v>
+        <v>16.48</v>
       </c>
       <c r="K17" s="4">
         <f>ROUND(I17*J17/100,2)</f>
@@ -13132,14 +13125,14 @@
         <v/>
       </c>
       <c r="M17" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N17" s="4">
         <f>ROUND(L17*M17,2)</f>
         <v/>
       </c>
       <c r="O17" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P17" s="4">
         <f>ROUND(N17*O17/100,2)</f>
@@ -13202,7 +13195,7 @@
         <v/>
       </c>
       <c r="J18" s="10" t="n">
-        <v>17</v>
+        <v>16.48</v>
       </c>
       <c r="K18" s="4">
         <f>ROUND(I18*J18/100,2)</f>
@@ -13213,14 +13206,14 @@
         <v/>
       </c>
       <c r="M18" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N18" s="4">
         <f>ROUND(L18*M18,2)</f>
         <v/>
       </c>
       <c r="O18" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P18" s="4">
         <f>ROUND(N18*O18/100,2)</f>
@@ -13283,7 +13276,7 @@
         <v/>
       </c>
       <c r="J19" s="10" t="n">
-        <v>16</v>
+        <v>15.59</v>
       </c>
       <c r="K19" s="4">
         <f>ROUND(I19*J19/100,2)</f>
@@ -13294,14 +13287,14 @@
         <v/>
       </c>
       <c r="M19" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N19" s="4">
         <f>ROUND(L19*M19,2)</f>
         <v/>
       </c>
       <c r="O19" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P19" s="4">
         <f>ROUND(N19*O19/100,2)</f>
@@ -13364,7 +13357,7 @@
         <v/>
       </c>
       <c r="J20" s="10" t="n">
-        <v>16</v>
+        <v>15.59</v>
       </c>
       <c r="K20" s="4">
         <f>ROUND(I20*J20/100,2)</f>
@@ -13375,14 +13368,14 @@
         <v/>
       </c>
       <c r="M20" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N20" s="4">
         <f>ROUND(L20*M20,2)</f>
         <v/>
       </c>
       <c r="O20" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P20" s="4">
         <f>ROUND(N20*O20/100,2)</f>
@@ -13445,7 +13438,7 @@
         <v/>
       </c>
       <c r="J21" s="10" t="n">
-        <v>15</v>
+        <v>14.76</v>
       </c>
       <c r="K21" s="4">
         <f>ROUND(I21*J21/100,2)</f>
@@ -13456,14 +13449,14 @@
         <v/>
       </c>
       <c r="M21" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N21" s="4">
         <f>ROUND(L21*M21,2)</f>
         <v/>
       </c>
       <c r="O21" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P21" s="4">
         <f>ROUND(N21*O21/100,2)</f>
@@ -13526,7 +13519,7 @@
         <v/>
       </c>
       <c r="J22" s="10" t="n">
-        <v>14</v>
+        <v>13.97</v>
       </c>
       <c r="K22" s="4">
         <f>ROUND(I22*J22/100,2)</f>
@@ -13537,14 +13530,14 @@
         <v/>
       </c>
       <c r="M22" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N22" s="4">
         <f>ROUND(L22*M22,2)</f>
         <v/>
       </c>
       <c r="O22" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P22" s="4">
         <f>ROUND(N22*O22/100,2)</f>
@@ -13607,7 +13600,7 @@
         <v/>
       </c>
       <c r="J23" s="10" t="n">
-        <v>13</v>
+        <v>13.06</v>
       </c>
       <c r="K23" s="4">
         <f>ROUND(I23*J23/100,2)</f>
@@ -13618,14 +13611,14 @@
         <v/>
       </c>
       <c r="M23" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N23" s="4">
         <f>ROUND(L23*M23,2)</f>
         <v/>
       </c>
       <c r="O23" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P23" s="4">
         <f>ROUND(N23*O23/100,2)</f>
@@ -13688,7 +13681,7 @@
         <v/>
       </c>
       <c r="J24" s="10" t="n">
-        <v>12</v>
+        <v>12.19</v>
       </c>
       <c r="K24" s="4">
         <f>ROUND(I24*J24/100,2)</f>
@@ -13699,14 +13692,14 @@
         <v/>
       </c>
       <c r="M24" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N24" s="4">
         <f>ROUND(L24*M24,2)</f>
         <v/>
       </c>
       <c r="O24" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P24" s="4">
         <f>ROUND(N24*O24/100,2)</f>
@@ -13769,7 +13762,7 @@
         <v/>
       </c>
       <c r="J25" s="10" t="n">
-        <v>11</v>
+        <v>11.35</v>
       </c>
       <c r="K25" s="4">
         <f>ROUND(I25*J25/100,2)</f>
@@ -13780,14 +13773,14 @@
         <v/>
       </c>
       <c r="M25" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N25" s="4">
         <f>ROUND(L25*M25,2)</f>
         <v/>
       </c>
       <c r="O25" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P25" s="4">
         <f>ROUND(N25*O25/100,2)</f>
@@ -13850,7 +13843,7 @@
         <v/>
       </c>
       <c r="J26" s="10" t="n">
-        <v>10</v>
+        <v>10.42</v>
       </c>
       <c r="K26" s="4">
         <f>ROUND(I26*J26/100,2)</f>
@@ -13861,14 +13854,14 @@
         <v/>
       </c>
       <c r="M26" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N26" s="4">
         <f>ROUND(L26*M26,2)</f>
         <v/>
       </c>
       <c r="O26" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P26" s="4">
         <f>ROUND(N26*O26/100,2)</f>
@@ -13931,7 +13924,7 @@
         <v/>
       </c>
       <c r="J27" s="10" t="n">
-        <v>9</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="K27" s="4">
         <f>ROUND(I27*J27/100,2)</f>
@@ -13942,14 +13935,14 @@
         <v/>
       </c>
       <c r="M27" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N27" s="4">
         <f>ROUND(L27*M27,2)</f>
         <v/>
       </c>
       <c r="O27" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P27" s="4">
         <f>ROUND(N27*O27/100,2)</f>
@@ -14012,7 +14005,7 @@
         <v/>
       </c>
       <c r="J28" s="10" t="n">
-        <v>8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="K28" s="4">
         <f>ROUND(I28*J28/100,2)</f>
@@ -14023,14 +14016,14 @@
         <v/>
       </c>
       <c r="M28" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N28" s="4">
         <f>ROUND(L28*M28,2)</f>
         <v/>
       </c>
       <c r="O28" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P28" s="4">
         <f>ROUND(N28*O28/100,2)</f>
@@ -14093,7 +14086,7 @@
         <v/>
       </c>
       <c r="J29" s="10" t="n">
-        <v>7</v>
+        <v>7.69</v>
       </c>
       <c r="K29" s="4">
         <f>ROUND(I29*J29/100,2)</f>
@@ -14104,14 +14097,14 @@
         <v/>
       </c>
       <c r="M29" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N29" s="4">
         <f>ROUND(L29*M29,2)</f>
         <v/>
       </c>
       <c r="O29" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P29" s="4">
         <f>ROUND(N29*O29/100,2)</f>
@@ -14174,7 +14167,7 @@
         <v/>
       </c>
       <c r="J30" s="10" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="K30" s="4">
         <f>ROUND(I30*J30/100,2)</f>
@@ -14185,14 +14178,14 @@
         <v/>
       </c>
       <c r="M30" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N30" s="4">
         <f>ROUND(L30*M30,2)</f>
         <v/>
       </c>
       <c r="O30" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P30" s="4">
         <f>ROUND(N30*O30/100,2)</f>
@@ -14255,7 +14248,7 @@
         <v/>
       </c>
       <c r="J31" s="10" t="n">
-        <v>5</v>
+        <v>5.74</v>
       </c>
       <c r="K31" s="4">
         <f>ROUND(I31*J31/100,2)</f>
@@ -14266,14 +14259,14 @@
         <v/>
       </c>
       <c r="M31" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N31" s="4">
         <f>ROUND(L31*M31,2)</f>
         <v/>
       </c>
       <c r="O31" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P31" s="4">
         <f>ROUND(N31*O31/100,2)</f>
@@ -14336,7 +14329,7 @@
         <v/>
       </c>
       <c r="J32" s="10" t="n">
-        <v>5</v>
+        <v>5.74</v>
       </c>
       <c r="K32" s="4">
         <f>ROUND(I32*J32/100,2)</f>
@@ -14347,14 +14340,14 @@
         <v/>
       </c>
       <c r="M32" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N32" s="4">
         <f>ROUND(L32*M32,2)</f>
         <v/>
       </c>
       <c r="O32" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P32" s="4">
         <f>ROUND(N32*O32/100,2)</f>
@@ -14417,7 +14410,7 @@
         <v/>
       </c>
       <c r="J33" s="10" t="n">
-        <v>4</v>
+        <v>4.68</v>
       </c>
       <c r="K33" s="4">
         <f>ROUND(I33*J33/100,2)</f>
@@ -14428,14 +14421,14 @@
         <v/>
       </c>
       <c r="M33" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N33" s="4">
         <f>ROUND(L33*M33,2)</f>
         <v/>
       </c>
       <c r="O33" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P33" s="4">
         <f>ROUND(N33*O33/100,2)</f>
@@ -14498,7 +14491,7 @@
         <v/>
       </c>
       <c r="J34" s="10" t="n">
-        <v>4</v>
+        <v>4.68</v>
       </c>
       <c r="K34" s="4">
         <f>ROUND(I34*J34/100,2)</f>
@@ -14509,14 +14502,14 @@
         <v/>
       </c>
       <c r="M34" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N34" s="4">
         <f>ROUND(L34*M34,2)</f>
         <v/>
       </c>
       <c r="O34" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P34" s="4">
         <f>ROUND(N34*O34/100,2)</f>
@@ -14579,7 +14572,7 @@
         <v/>
       </c>
       <c r="J35" s="10" t="n">
-        <v>3</v>
+        <v>3.54</v>
       </c>
       <c r="K35" s="4">
         <f>ROUND(I35*J35/100,2)</f>
@@ -14590,14 +14583,14 @@
         <v/>
       </c>
       <c r="M35" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N35" s="4">
         <f>ROUND(L35*M35,2)</f>
         <v/>
       </c>
       <c r="O35" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P35" s="4">
         <f>ROUND(N35*O35/100,2)</f>
@@ -14660,7 +14653,7 @@
         <v/>
       </c>
       <c r="J36" s="10" t="n">
-        <v>2</v>
+        <v>2.44</v>
       </c>
       <c r="K36" s="4">
         <f>ROUND(I36*J36/100,2)</f>
@@ -14671,14 +14664,14 @@
         <v/>
       </c>
       <c r="M36" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N36" s="4">
         <f>ROUND(L36*M36,2)</f>
         <v/>
       </c>
       <c r="O36" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P36" s="4">
         <f>ROUND(N36*O36/100,2)</f>
@@ -14741,7 +14734,7 @@
         <v/>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1</v>
+        <v>1.16</v>
       </c>
       <c r="K37" s="4">
         <f>ROUND(I37*J37/100,2)</f>
@@ -14752,14 +14745,14 @@
         <v/>
       </c>
       <c r="M37" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N37" s="4">
         <f>ROUND(L37*M37,2)</f>
         <v/>
       </c>
       <c r="O37" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P37" s="4">
         <f>ROUND(N37*O37/100,2)</f>
@@ -14833,14 +14826,14 @@
         <v/>
       </c>
       <c r="M38" s="17" t="n">
-        <v>1.0490702075</v>
+        <v>1.0398329699</v>
       </c>
       <c r="N38" s="4">
         <f>ROUND(L38*M38,2)</f>
         <v/>
       </c>
       <c r="O38" s="10" t="n">
-        <v>7.2</v>
+        <v>9.81</v>
       </c>
       <c r="P38" s="4">
         <f>ROUND(N38*O38/100,2)</f>
@@ -14914,14 +14907,14 @@
         <v/>
       </c>
       <c r="M39" s="17" t="n">
-        <v>1.044890645</v>
+        <v>1.0344538101</v>
       </c>
       <c r="N39" s="4">
         <f>ROUND(L39*M39,2)</f>
         <v/>
       </c>
       <c r="O39" s="10" t="n">
-        <v>6.6</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="P39" s="4">
         <f>ROUND(N39*O39/100,2)</f>
@@ -14995,14 +14988,14 @@
         <v/>
       </c>
       <c r="M40" s="17" t="n">
-        <v>1.040727734</v>
+        <v>1.0341435671</v>
       </c>
       <c r="N40" s="4">
         <f>ROUND(L40*M40,2)</f>
         <v/>
       </c>
       <c r="O40" s="10" t="n">
-        <v>6</v>
+        <v>7.86</v>
       </c>
       <c r="P40" s="4">
         <f>ROUND(N40*O40/100,2)</f>
@@ -15076,14 +15069,14 @@
         <v/>
       </c>
       <c r="M41" s="17" t="n">
-        <v>1.0365814084</v>
+        <v>1.033833417</v>
       </c>
       <c r="N41" s="4">
         <f>ROUND(L41*M41,2)</f>
         <v/>
       </c>
       <c r="O41" s="10" t="n">
-        <v>5.4</v>
+        <v>6.84</v>
       </c>
       <c r="P41" s="4">
         <f>ROUND(N41*O41/100,2)</f>
@@ -15157,14 +15150,14 @@
         <v/>
       </c>
       <c r="M42" s="17" t="n">
-        <v>1.032451602</v>
+        <v>1.0316669165</v>
       </c>
       <c r="N42" s="4">
         <f>ROUND(L42*M42,2)</f>
         <v/>
       </c>
       <c r="O42" s="10" t="n">
-        <v>4.8</v>
+        <v>5.83</v>
       </c>
       <c r="P42" s="4">
         <f>ROUND(N42*O42/100,2)</f>
@@ -15238,14 +15231,14 @@
         <v/>
       </c>
       <c r="M43" s="17" t="n">
-        <v>1.028338249</v>
+        <v>1.0276590462</v>
       </c>
       <c r="N43" s="4">
         <f>ROUND(L43*M43,2)</f>
         <v/>
       </c>
       <c r="O43" s="10" t="n">
-        <v>4.2</v>
+        <v>5.06</v>
       </c>
       <c r="P43" s="4">
         <f>ROUND(N43*O43/100,2)</f>
@@ -15319,14 +15312,14 @@
         <v/>
       </c>
       <c r="M44" s="17" t="n">
-        <v>1.0242412838</v>
+        <v>1.0219362035</v>
       </c>
       <c r="N44" s="4">
         <f>ROUND(L44*M44,2)</f>
         <v/>
       </c>
       <c r="O44" s="10" t="n">
-        <v>3.6</v>
+        <v>4.62</v>
       </c>
       <c r="P44" s="4">
         <f>ROUND(N44*O44/100,2)</f>
@@ -15400,14 +15393,14 @@
         <v/>
       </c>
       <c r="M45" s="17" t="n">
-        <v>1.0201606413</v>
+        <v>1.0127204474</v>
       </c>
       <c r="N45" s="4">
         <f>ROUND(L45*M45,2)</f>
         <v/>
       </c>
       <c r="O45" s="10" t="n">
-        <v>3</v>
+        <v>4.32</v>
       </c>
       <c r="P45" s="4">
         <f>ROUND(N45*O45/100,2)</f>
@@ -15481,14 +15474,14 @@
         <v/>
       </c>
       <c r="M46" s="17" t="n">
-        <v>1.0201606413</v>
+        <v>1.0127204474</v>
       </c>
       <c r="N46" s="4">
         <f>ROUND(L46*M46,2)</f>
         <v/>
       </c>
       <c r="O46" s="10" t="n">
-        <v>3</v>
+        <v>4.32</v>
       </c>
       <c r="P46" s="4">
         <f>ROUND(N46*O46/100,2)</f>
@@ -15562,14 +15555,14 @@
         <v/>
       </c>
       <c r="M47" s="17" t="n">
-        <v>1.0160962563</v>
+        <v>1.0045833225</v>
       </c>
       <c r="N47" s="4">
         <f>ROUND(L47*M47,2)</f>
         <v/>
       </c>
       <c r="O47" s="10" t="n">
-        <v>2.4</v>
+        <v>4.04</v>
       </c>
       <c r="P47" s="4">
         <f>ROUND(N47*O47/100,2)</f>
@@ -15643,14 +15636,14 @@
         <v/>
       </c>
       <c r="M48" s="17" t="n">
-        <v>1.0160962563</v>
+        <v>1.0045833225</v>
       </c>
       <c r="N48" s="4">
         <f>ROUND(L48*M48,2)</f>
         <v/>
       </c>
       <c r="O48" s="10" t="n">
-        <v>2.4</v>
+        <v>4.04</v>
       </c>
       <c r="P48" s="4">
         <f>ROUND(N48*O48/100,2)</f>
@@ -15724,14 +15717,14 @@
         <v/>
       </c>
       <c r="M49" s="17" t="n">
-        <v>1.012048064</v>
+        <v>0.9980957004</v>
       </c>
       <c r="N49" s="4">
         <f>ROUND(L49*M49,2)</f>
         <v/>
       </c>
       <c r="O49" s="10" t="n">
-        <v>1.8</v>
+        <v>3.62</v>
       </c>
       <c r="P49" s="4">
         <f>ROUND(N49*O49/100,2)</f>
@@ -15805,14 +15798,14 @@
         <v/>
       </c>
       <c r="M50" s="17" t="n">
-        <v>1.008016</v>
+        <v>0.99670032</v>
       </c>
       <c r="N50" s="4">
         <f>ROUND(L50*M50,2)</f>
         <v/>
       </c>
       <c r="O50" s="10" t="n">
-        <v>1.2</v>
+        <v>2.64</v>
       </c>
       <c r="P50" s="4">
         <f>ROUND(N50*O50/100,2)</f>
@@ -15886,14 +15879,14 @@
         <v/>
       </c>
       <c r="M51" s="17" t="n">
-        <v>1.004</v>
+        <v>0.9968</v>
       </c>
       <c r="N51" s="4">
         <f>ROUND(L51*M51,2)</f>
         <v/>
       </c>
       <c r="O51" s="10" t="n">
-        <v>0.6</v>
+        <v>1.41</v>
       </c>
       <c r="P51" s="4">
         <f>ROUND(N51*O51/100,2)</f>

</xml_diff>